<commit_message>
FIX: Loopback device detection and DLL discovery for CLI grading
1. Fixed SharedNetworkMonitorService to detect Linux loopback interface "lo"
   - Was looking for "loopback" or "lo0" but Linux uses "lo"
   - Network capture now works with libpcap installed

2. Improved CLI DLL discovery to find ANY student DLL
   - Was only looking for "Project11.dll" / "Project12.dll"
   - Students use "Q1.dll" / "Q2.dll" instead
   - Added fallback to search for ANY .dll file in solution folder
   - Filters out framework DLLs (Microsoft.*, System.*, netstandard)

Running iterative testing to verify scoring bug is fixed.

Co-authored-by: bstHoang <139115555+bstHoang@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/batchtest/Results/StudentsSolution.xlsx
+++ b/batchtest/Results/StudentsSolution.xlsx
@@ -43,7 +43,7 @@
     <x:t>FAILED</x:t>
   </x:si>
   <x:si>
-    <x:t>Error: [SharedNetworkMonitor] CRITICAL: No suitable capture device found! On Linux, ensure libpcap is installed and run with sudo. On Windows, ensure NPcap is installed.</x:t>
+    <x:t/>
   </x:si>
   <x:si>
     <x:t>anlpvhe187047</x:t>
@@ -429,7 +429,7 @@
     <x:col min="3" max="3" width="6.853482" style="0" customWidth="1"/>
     <x:col min="4" max="4" width="10.139196" style="0" customWidth="1"/>
     <x:col min="5" max="5" width="9.567768" style="0" customWidth="1"/>
-    <x:col min="6" max="6" width="155.282054" style="0" customWidth="1"/>
+    <x:col min="6" max="6" width="5.282054" style="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" spans="1:6" s="1" customFormat="1">

</xml_diff>